<commit_message>
Refresh FR data as of July 28
</commit_message>
<xml_diff>
--- a/data/fr/FR_Budget_Status.xlsx
+++ b/data/fr/FR_Budget_Status.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\WR\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12315"/>
   </bookViews>
   <sheets>
     <sheet name="OPEN LINE FR" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="48">
   <si>
     <t>Plan Head</t>
   </si>
@@ -163,9 +163,6 @@
     <t>SBA 2026-27</t>
   </si>
   <si>
-    <t>22.06.2026</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -187,7 +184,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Actual.  Expenditure of Demand 16 upto as on  30.06.2026  (Fig.in Thousand) </t>
+      <t xml:space="preserve">Actual.  Expenditure of Demand 16 upto as on  28.07.2026  (Fig.in Thousand) </t>
     </r>
     <r>
       <rPr>
@@ -223,7 +220,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Actual.  Expenditure of Demand 16 GSU as on  30.06.2026  (Fig.in Thousand)</t>
+      <t>Actual.  Expenditure of Demand 16 GSU as on  28.07.2026  (Fig.in Thousand)</t>
     </r>
     <r>
       <rPr>
@@ -3048,7 +3045,7 @@
   <sheetData>
     <row r="1" spans="1:244" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
@@ -3216,11 +3213,11 @@
         <v>146190</v>
       </c>
       <c r="D4" s="13">
-        <v>26053</v>
+        <v>48449</v>
       </c>
       <c r="E4" s="14">
         <f>D4-C4</f>
-        <v>-120137</v>
+        <v>-97741</v>
       </c>
       <c r="F4" s="11">
         <v>0</v>
@@ -3288,15 +3285,15 @@
       </c>
       <c r="Y4" s="13">
         <f t="shared" si="3"/>
-        <v>26747</v>
+        <v>49143</v>
       </c>
       <c r="Z4" s="14">
         <f>Y4-X4</f>
-        <v>-134156</v>
+        <v>-111760</v>
       </c>
       <c r="AA4" s="6">
         <f>Y4/X4*100</f>
-        <v>16.623058612953145</v>
+        <v>30.542003567366677</v>
       </c>
       <c r="AB4"/>
       <c r="AC4"/>
@@ -3383,11 +3380,11 @@
         <v>4107</v>
       </c>
       <c r="D5" s="6">
-        <v>2511</v>
+        <v>2818</v>
       </c>
       <c r="E5" s="14">
         <f t="shared" ref="E5:E21" si="4">D5-C5</f>
-        <v>-1596</v>
+        <v>-1289</v>
       </c>
       <c r="F5" s="5">
         <v>14120</v>
@@ -3455,15 +3452,15 @@
       </c>
       <c r="Y5" s="13">
         <f t="shared" si="3"/>
-        <v>3375</v>
+        <v>3682</v>
       </c>
       <c r="Z5" s="14">
         <f t="shared" ref="Z5:Z21" si="8">Y5-X5</f>
-        <v>-28852</v>
+        <v>-28545</v>
       </c>
       <c r="AA5" s="6">
         <f t="shared" ref="AA5:AA20" si="9">Y5/X5*100</f>
-        <v>10.472585099450772</v>
+        <v>11.425202469978588</v>
       </c>
     </row>
     <row r="6" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3517,11 +3514,11 @@
         <v>120318</v>
       </c>
       <c r="P6" s="8">
-        <v>45115</v>
+        <v>49669</v>
       </c>
       <c r="Q6" s="14">
         <f t="shared" si="7"/>
-        <v>-75203</v>
+        <v>-70649</v>
       </c>
       <c r="R6" s="14">
         <v>0</v>
@@ -3549,15 +3546,15 @@
       </c>
       <c r="Y6" s="13">
         <f t="shared" si="3"/>
-        <v>45115</v>
+        <v>49669</v>
       </c>
       <c r="Z6" s="14">
         <f t="shared" si="8"/>
-        <v>-75203</v>
+        <v>-70649</v>
       </c>
       <c r="AA6" s="6">
         <f t="shared" si="9"/>
-        <v>37.496467693944382</v>
+        <v>41.281437523895008</v>
       </c>
     </row>
     <row r="7" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3611,11 +3608,11 @@
         <v>316420</v>
       </c>
       <c r="P7" s="8">
-        <v>194943</v>
+        <v>221758</v>
       </c>
       <c r="Q7" s="14">
         <f t="shared" si="7"/>
-        <v>-121477</v>
+        <v>-94662</v>
       </c>
       <c r="R7" s="7">
         <v>0</v>
@@ -3631,11 +3628,11 @@
         <v>191000</v>
       </c>
       <c r="V7" s="6">
-        <v>85138</v>
+        <v>92917</v>
       </c>
       <c r="W7" s="14">
         <f t="shared" si="2"/>
-        <v>-105862</v>
+        <v>-98083</v>
       </c>
       <c r="X7" s="12">
         <f t="shared" si="3"/>
@@ -3643,15 +3640,15 @@
       </c>
       <c r="Y7" s="13">
         <f t="shared" si="3"/>
-        <v>280081</v>
+        <v>314675</v>
       </c>
       <c r="Z7" s="14">
         <f t="shared" si="8"/>
-        <v>-227339</v>
+        <v>-192745</v>
       </c>
       <c r="AA7" s="6">
         <f t="shared" si="9"/>
-        <v>55.197075401048444</v>
+        <v>62.01470182491822</v>
       </c>
     </row>
     <row r="8" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3705,11 +3702,11 @@
         <v>2645397</v>
       </c>
       <c r="P8" s="8">
-        <v>2131498</v>
+        <v>2172711</v>
       </c>
       <c r="Q8" s="14">
         <f t="shared" si="7"/>
-        <v>-513899</v>
+        <v>-472686</v>
       </c>
       <c r="R8" s="7">
         <v>0</v>
@@ -3725,11 +3722,11 @@
         <v>317398</v>
       </c>
       <c r="V8" s="6">
-        <v>178422</v>
+        <v>183459</v>
       </c>
       <c r="W8" s="14">
         <f t="shared" si="2"/>
-        <v>-138976</v>
+        <v>-133939</v>
       </c>
       <c r="X8" s="12">
         <f t="shared" si="3"/>
@@ -3737,15 +3734,15 @@
       </c>
       <c r="Y8" s="13">
         <f t="shared" si="3"/>
-        <v>2309920</v>
+        <v>2356170</v>
       </c>
       <c r="Z8" s="14">
         <f t="shared" si="8"/>
-        <v>-652875</v>
+        <v>-606625</v>
       </c>
       <c r="AA8" s="6">
         <f t="shared" si="9"/>
-        <v>77.964219596698399</v>
+        <v>79.525245587359223</v>
       </c>
     </row>
     <row r="9" spans="1:244" s="4" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3799,11 +3796,11 @@
         <v>35380</v>
       </c>
       <c r="P9" s="15">
-        <v>14445</v>
+        <v>19188</v>
       </c>
       <c r="Q9" s="14">
         <f t="shared" si="7"/>
-        <v>-20935</v>
+        <v>-16192</v>
       </c>
       <c r="R9" s="14">
         <v>0</v>
@@ -3819,11 +3816,11 @@
         <v>96867</v>
       </c>
       <c r="V9" s="13">
-        <v>103026</v>
+        <v>116765</v>
       </c>
       <c r="W9" s="14">
         <f t="shared" si="2"/>
-        <v>6159</v>
+        <v>19898</v>
       </c>
       <c r="X9" s="12">
         <f t="shared" si="3"/>
@@ -3831,15 +3828,15 @@
       </c>
       <c r="Y9" s="13">
         <f t="shared" si="3"/>
-        <v>117471</v>
+        <v>135953</v>
       </c>
       <c r="Z9" s="14">
         <f t="shared" si="8"/>
-        <v>-14796</v>
+        <v>3686</v>
       </c>
       <c r="AA9" s="6">
         <f t="shared" si="9"/>
-        <v>88.813536256209034</v>
+        <v>102.78678733168516</v>
       </c>
       <c r="AB9"/>
       <c r="AC9"/>
@@ -4070,11 +4067,11 @@
         <v>159700</v>
       </c>
       <c r="D10" s="13">
-        <v>7634</v>
+        <v>8146</v>
       </c>
       <c r="E10" s="14">
         <f t="shared" si="4"/>
-        <v>-152066</v>
+        <v>-151554</v>
       </c>
       <c r="F10" s="12">
         <v>0</v>
@@ -4130,11 +4127,11 @@
         <v>363143</v>
       </c>
       <c r="V10" s="13">
-        <v>76152</v>
+        <v>109527</v>
       </c>
       <c r="W10" s="14">
         <f t="shared" si="2"/>
-        <v>-286991</v>
+        <v>-253616</v>
       </c>
       <c r="X10" s="12">
         <f t="shared" si="3"/>
@@ -4142,15 +4139,15 @@
       </c>
       <c r="Y10" s="13">
         <f t="shared" si="3"/>
-        <v>83786</v>
+        <v>117673</v>
       </c>
       <c r="Z10" s="14">
         <f t="shared" si="8"/>
-        <v>-439057</v>
+        <v>-405170</v>
       </c>
       <c r="AA10" s="6">
         <f t="shared" si="9"/>
-        <v>16.025078273975172</v>
+        <v>22.506373806286017</v>
       </c>
       <c r="AB10"/>
       <c r="AC10"/>
@@ -4381,11 +4378,11 @@
         <v>174056</v>
       </c>
       <c r="D11" s="6">
-        <v>65941</v>
+        <v>70459</v>
       </c>
       <c r="E11" s="14">
         <f t="shared" si="4"/>
-        <v>-108115</v>
+        <v>-103597</v>
       </c>
       <c r="F11" s="5">
         <v>0</v>
@@ -4441,11 +4438,11 @@
         <v>107957</v>
       </c>
       <c r="V11" s="6">
-        <v>11777</v>
+        <v>11903</v>
       </c>
       <c r="W11" s="14">
         <f t="shared" si="2"/>
-        <v>-96180</v>
+        <v>-96054</v>
       </c>
       <c r="X11" s="12">
         <f t="shared" si="3"/>
@@ -4453,15 +4450,15 @@
       </c>
       <c r="Y11" s="13">
         <f t="shared" si="3"/>
-        <v>77718</v>
+        <v>82362</v>
       </c>
       <c r="Z11" s="14">
         <f t="shared" si="8"/>
-        <v>-230125</v>
+        <v>-225481</v>
       </c>
       <c r="AA11" s="6">
         <f t="shared" si="9"/>
-        <v>25.245985778464998</v>
+        <v>26.754546960626037</v>
       </c>
     </row>
     <row r="12" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4569,11 +4566,11 @@
         <v>10884</v>
       </c>
       <c r="D13" s="6">
-        <v>282</v>
+        <v>1983</v>
       </c>
       <c r="E13" s="14">
         <f t="shared" si="4"/>
-        <v>-10602</v>
+        <v>-8901</v>
       </c>
       <c r="F13" s="5">
         <v>1</v>
@@ -4629,11 +4626,11 @@
         <v>2000</v>
       </c>
       <c r="V13" s="6">
-        <v>1637</v>
+        <v>1646</v>
       </c>
       <c r="W13" s="14">
         <f t="shared" si="2"/>
-        <v>-363</v>
+        <v>-354</v>
       </c>
       <c r="X13" s="12">
         <f t="shared" si="3"/>
@@ -4641,15 +4638,15 @@
       </c>
       <c r="Y13" s="13">
         <f t="shared" si="3"/>
-        <v>1919</v>
+        <v>3629</v>
       </c>
       <c r="Z13" s="14">
         <f t="shared" si="8"/>
-        <v>-11275</v>
+        <v>-9565</v>
       </c>
       <c r="AA13" s="6">
         <f t="shared" si="9"/>
-        <v>14.544489919660453</v>
+        <v>27.50492648173412</v>
       </c>
     </row>
     <row r="14" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4663,11 +4660,11 @@
         <v>35702</v>
       </c>
       <c r="D14" s="6">
-        <v>2426</v>
+        <v>2427</v>
       </c>
       <c r="E14" s="14">
         <f t="shared" si="4"/>
-        <v>-33276</v>
+        <v>-33275</v>
       </c>
       <c r="F14" s="5">
         <v>2000</v>
@@ -4735,15 +4732,15 @@
       </c>
       <c r="Y14" s="13">
         <f t="shared" si="3"/>
-        <v>2426</v>
+        <v>2427</v>
       </c>
       <c r="Z14" s="14">
         <f t="shared" si="8"/>
-        <v>-51276</v>
+        <v>-51275</v>
       </c>
       <c r="AA14" s="6">
         <f t="shared" si="9"/>
-        <v>4.517522624855685</v>
+        <v>4.5193847528956086</v>
       </c>
     </row>
     <row r="15" spans="1:244" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4757,11 +4754,11 @@
         <v>62500</v>
       </c>
       <c r="D15" s="6">
-        <v>18119</v>
+        <v>31212</v>
       </c>
       <c r="E15" s="14">
         <f t="shared" si="4"/>
-        <v>-44381</v>
+        <v>-31288</v>
       </c>
       <c r="F15" s="5">
         <v>12000</v>
@@ -4829,15 +4826,15 @@
       </c>
       <c r="Y15" s="13">
         <f t="shared" si="3"/>
-        <v>22047</v>
+        <v>35140</v>
       </c>
       <c r="Z15" s="14">
         <f t="shared" si="8"/>
-        <v>-75453</v>
+        <v>-62360</v>
       </c>
       <c r="AA15" s="6">
         <f t="shared" si="9"/>
-        <v>22.612307692307692</v>
+        <v>36.041025641025641</v>
       </c>
     </row>
     <row r="16" spans="1:244" s="4" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -4851,11 +4848,11 @@
         <v>285610</v>
       </c>
       <c r="D16" s="13">
-        <v>120402</v>
+        <v>109952</v>
       </c>
       <c r="E16" s="14">
         <f t="shared" si="4"/>
-        <v>-165208</v>
+        <v>-175658</v>
       </c>
       <c r="F16" s="12">
         <v>0</v>
@@ -4923,15 +4920,15 @@
       </c>
       <c r="Y16" s="13">
         <f t="shared" si="3"/>
-        <v>125504</v>
+        <v>115054</v>
       </c>
       <c r="Z16" s="14">
         <f t="shared" si="8"/>
-        <v>-185408</v>
+        <v>-195858</v>
       </c>
       <c r="AA16" s="6">
         <f t="shared" si="9"/>
-        <v>40.366405928365587</v>
+        <v>37.005326265953066</v>
       </c>
       <c r="AB16"/>
       <c r="AC16"/>
@@ -5130,11 +5127,11 @@
         <v>69550</v>
       </c>
       <c r="D18" s="13">
-        <v>19043</v>
+        <v>21544</v>
       </c>
       <c r="E18" s="14">
         <f t="shared" si="4"/>
-        <v>-50507</v>
+        <v>-48006</v>
       </c>
       <c r="F18" s="12">
         <v>12111</v>
@@ -5150,11 +5147,11 @@
         <v>62003</v>
       </c>
       <c r="J18" s="13">
-        <v>6208</v>
+        <v>6804</v>
       </c>
       <c r="K18" s="14">
         <f t="shared" si="5"/>
-        <v>-55795</v>
+        <v>-55199</v>
       </c>
       <c r="L18" s="14">
         <v>0</v>
@@ -5190,11 +5187,11 @@
         <v>172069</v>
       </c>
       <c r="V18" s="29">
-        <v>38247</v>
+        <v>38637</v>
       </c>
       <c r="W18" s="14">
         <f t="shared" si="2"/>
-        <v>-133822</v>
+        <v>-133432</v>
       </c>
       <c r="X18" s="12">
         <f t="shared" si="3"/>
@@ -5202,15 +5199,15 @@
       </c>
       <c r="Y18" s="13">
         <f t="shared" si="3"/>
-        <v>71352</v>
+        <v>74839</v>
       </c>
       <c r="Z18" s="14">
         <f t="shared" si="8"/>
-        <v>-244381</v>
+        <v>-240894</v>
       </c>
       <c r="AA18" s="6">
         <f>Y18/X18*100</f>
-        <v>22.598841426141707</v>
+        <v>23.703255598876265</v>
       </c>
       <c r="AB18"/>
       <c r="AC18"/>
@@ -6859,11 +6856,11 @@
       </c>
       <c r="D21" s="1">
         <f>SUM(D4:D20)</f>
-        <v>262411</v>
+        <v>296990</v>
       </c>
       <c r="E21" s="14">
         <f t="shared" si="4"/>
-        <v>-755942</v>
+        <v>-721363</v>
       </c>
       <c r="F21" s="2">
         <f>SUM(F4:F20)</f>
@@ -6883,11 +6880,11 @@
       </c>
       <c r="J21" s="1">
         <f>SUM(J4:J20)</f>
-        <v>8107</v>
+        <v>8703</v>
       </c>
       <c r="K21" s="14">
         <f t="shared" si="5"/>
-        <v>-122485</v>
+        <v>-121889</v>
       </c>
       <c r="L21" s="2">
         <f>SUM(L4:L20)</f>
@@ -6907,11 +6904,11 @@
       </c>
       <c r="P21" s="1">
         <f>SUM(P4:P20)</f>
-        <v>2386001</v>
+        <v>2463326</v>
       </c>
       <c r="Q21" s="14">
         <f t="shared" si="7"/>
-        <v>-731514</v>
+        <v>-654189</v>
       </c>
       <c r="R21" s="1">
         <f>SUM(R4:R20)</f>
@@ -6931,11 +6928,11 @@
       </c>
       <c r="V21" s="1">
         <f>SUM(V4:V20)</f>
-        <v>498296</v>
+        <v>558751</v>
       </c>
       <c r="W21" s="7">
         <f t="shared" si="2"/>
-        <v>-802713</v>
+        <v>-742258</v>
       </c>
       <c r="X21" s="12">
         <f t="shared" si="13"/>
@@ -6943,18 +6940,15 @@
       </c>
       <c r="Y21" s="13">
         <f t="shared" si="13"/>
-        <v>3167461</v>
+        <v>3340416</v>
       </c>
       <c r="Z21" s="14">
         <f t="shared" si="8"/>
-        <v>-2440240</v>
+        <v>-2267285</v>
       </c>
       <c r="AA21" s="6">
         <f>Y21/X21*100</f>
-        <v>56.484127809239467</v>
-      </c>
-      <c r="AC21" t="s">
-        <v>46</v>
+        <v>59.568368570292883</v>
       </c>
     </row>
     <row r="22" spans="1:1476" x14ac:dyDescent="0.25">
@@ -7854,7 +7848,7 @@
   <sheetData>
     <row r="1" spans="1:35" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="51" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" s="51"/>
       <c r="C1" s="51"/>
@@ -8373,11 +8367,11 @@
         <v>1</v>
       </c>
       <c r="V7" s="6">
-        <v>0.69799999999999995</v>
+        <v>127</v>
       </c>
       <c r="W7" s="7">
         <f t="shared" si="10"/>
-        <v>-0.30200000000000005</v>
+        <v>126</v>
       </c>
       <c r="X7" s="5">
         <f t="shared" si="0"/>
@@ -8385,15 +8379,15 @@
       </c>
       <c r="Y7" s="6">
         <f t="shared" si="7"/>
-        <v>0.69799999999999995</v>
+        <v>127</v>
       </c>
       <c r="Z7" s="7">
         <f t="shared" si="8"/>
-        <v>-0.30200000000000005</v>
+        <v>126</v>
       </c>
       <c r="AA7" s="6">
         <f t="shared" ref="AA7:AA21" si="11">Y7/X7*100</f>
-        <v>69.8</v>
+        <v>12700</v>
       </c>
     </row>
     <row r="8" spans="1:35" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -8966,11 +8960,11 @@
         <v>5001</v>
       </c>
       <c r="D14" s="6">
-        <v>0</v>
+        <v>2048</v>
       </c>
       <c r="E14" s="7">
         <f t="shared" si="2"/>
-        <v>-5001</v>
+        <v>-2953</v>
       </c>
       <c r="F14" s="5">
         <v>0</v>
@@ -9038,15 +9032,15 @@
       </c>
       <c r="Y14" s="6">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2048</v>
       </c>
       <c r="Z14" s="7">
         <f t="shared" si="8"/>
-        <v>-5001</v>
+        <v>-2953</v>
       </c>
       <c r="AA14" s="6">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>40.951809638072383</v>
       </c>
     </row>
     <row r="15" spans="1:35" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -9151,11 +9145,11 @@
         <v>446600</v>
       </c>
       <c r="D16" s="6">
-        <v>198329</v>
+        <v>239160</v>
       </c>
       <c r="E16" s="7">
         <f t="shared" si="2"/>
-        <v>-248271</v>
+        <v>-207440</v>
       </c>
       <c r="F16" s="5">
         <v>0</v>
@@ -9223,15 +9217,15 @@
       </c>
       <c r="Y16" s="6">
         <f t="shared" si="7"/>
-        <v>198329</v>
+        <v>239160</v>
       </c>
       <c r="Z16" s="7">
         <f t="shared" si="8"/>
-        <v>-248271</v>
+        <v>-207440</v>
       </c>
       <c r="AA16" s="6">
         <f t="shared" si="11"/>
-        <v>44.408643081056873</v>
+        <v>53.551276309896998</v>
       </c>
     </row>
     <row r="17" spans="1:34" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -9618,11 +9612,11 @@
       </c>
       <c r="D21" s="1">
         <f>SUM(D4:D20)</f>
-        <v>198329</v>
+        <v>241208</v>
       </c>
       <c r="E21" s="7">
         <f t="shared" ref="E21" si="20">D21-C21</f>
-        <v>-253272</v>
+        <v>-210393</v>
       </c>
       <c r="F21" s="2">
         <f>SUM(F4:F20)</f>
@@ -9689,11 +9683,11 @@
       </c>
       <c r="V21" s="1">
         <f>SUM(V4:V20)</f>
-        <v>0.69799999999999995</v>
+        <v>127</v>
       </c>
       <c r="W21" s="7">
         <f>V21-U21</f>
-        <v>-0.30200000000000005</v>
+        <v>126</v>
       </c>
       <c r="X21" s="5">
         <f t="shared" si="19"/>
@@ -9701,15 +9695,15 @@
       </c>
       <c r="Y21" s="6">
         <f t="shared" si="7"/>
-        <v>198329.698</v>
+        <v>241335</v>
       </c>
       <c r="Z21" s="7">
         <f t="shared" si="8"/>
-        <v>-253273.302</v>
+        <v>-210268</v>
       </c>
       <c r="AA21" s="6">
         <f t="shared" si="11"/>
-        <v>43.916824733228076</v>
+        <v>53.439636140592519</v>
       </c>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">

</xml_diff>